<commit_message>
Add app install auth tests, BLE/start/stop evidence, Gen2X docs, and 07 Sep findings
- Expand .gitignore to exclude private keys, cert bundles, PFX files, and the
  local Python venv from future commits.
- Add app install authentication test requests (basic, bearer, mtls, none) and
  further BLE config, start/stop, and impinjGen2X PUT test evidence.
- Add Gen2x documentation.json, the 07 Sep findings workbook, and the scripts
  used to generate/trim it.
- Refresh MQTT and REST examples across many endpoints, and rebuild the
  generated MQTT/REST specs to match.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/captures/FXR-API-Findings-For-Developer_2026-09-01.xlsx
+++ b/captures/FXR-API-Findings-For-Developer_2026-09-01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Questions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Questions'!$A$2:$H$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Questions'!$A$2:$H$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -44,7 +44,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -72,8 +72,18 @@
         <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -96,11 +106,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -118,6 +134,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -485,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1319,8 +1341,116 @@
         </is>
       </c>
     </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="7" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>PUT /cloud/mode</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>set_mode</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>wordCounter vs wordCount</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>wordCount works in the READ access config. wordCounter is rejected (HTTP 422): "wordCount must be included in access-config object for read". After renaming the field, TID is returned in accessResults.</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>The READ config requires wordCounter. The with_accesses example also uses wordCounter. MQTT set_mode uses the same name. The description on wordCounter repeats "WordPtr Field" (that is wordPointer).</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>Can you change the spec field name from wordCounter to wordCount so it matches the reader?</t>
+        </is>
+      </c>
+      <c r="H25" s="8" t="n"/>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>PUT /cloud/bleConfig (GET /cloud/bleConfig response: generic filters)</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>set_bleConfig / get_bleConfig</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>generic filter field casing</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>The generic filter accepts only lowercase names: address, addressType, name, alias. Capital names Address, AddressType, Name, Alias are rejected (HTTP 422): unknown or unexpected field. Isolated by bisection on reader 5.0.7. After lowercasing, the same body is stored and read back.</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>PUT schema, PUT example enable_with_protocols, and GET schema/example all use Address, AddressType, Name, Alias. Those look like BLE output event names pasted into the input filter.</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Can you change the generic filter field names to address, addressType, name, alias in both the schema and the examples (PUT enable_with_protocols and GET)? Same names appear on GET /cloud/bleConfig.</t>
+        </is>
+      </c>
+      <c r="H26" s="8" t="n"/>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>PUT /cloud/bleConfig</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>set_bleConfig</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>four required ble fields vs description / short examples</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>PUT fails if any of these four is missing: enable, scanIntervalSec, protocols, additionalFilters. A short body such as {"ble":{"enable":true}} is rejected. additionalFilters may be {}. protocols may list only one protocol. All four keys must still be present.</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>The schema required list already has those four fields. The operation description still says only ble.enable is required and the other fields are optional. That wording does not match the schema or the reader.</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>Can you change the description so it says all four fields are required (enable, scanIntervalSec, protocols, additionalFilters), matching the schema and the reader? Please also check that no example omits any of the four — a short example will fail on the device.</t>
+        </is>
+      </c>
+      <c r="H27" s="8" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:H24"/>
+  <autoFilter ref="A2:H25"/>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>
   </mergeCells>

</xml_diff>